<commit_message>
Servicio con 3 personas y menú vegetariano; script de validación
- Supuestos v0.8: S15 (21 s por ración), S22 (3 sirviendo, una a cargo del menú
  vegetariano), S13 corregido, S27 nuevo (12 % vegetarianos), D06 a redefinir.
- inputs.xlsx: Escenarios con ProbVegetariano (reemplaza FilasPorTipo), E4 y E5 con 4
  sirviendo, TiemposServicio actualizado.
- referencia_modelo.py: una sola fila de caja y puesto vegetariano en el mostrador.
- validar_modelo.py: valida una corrida de FlexSim contra la realidad y contra la réplica.
- GUIA_MODIFICACIONES.md: pasos para aplicar el cambio en el modelo de FlexSim.
- AVANCE.md con la etapa A probada; modelo comedor_unc_1.fsm; el modelo anterior queda en
  flexsim/Obsoleto. flexsim/salidas.xlsx es una exportación previa al cambio.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/flexsim/inputs.xlsx
+++ b/flexsim/inputs.xlsx
@@ -464,7 +464,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado por analisis/generar_inputs_flexsim.py a partir de supuestos/supuestos.json v0.7. No editar a mano: cambiar el JSON y regenerar.</t>
+          <t>Generado por analisis/generar_inputs_flexsim.py a partir de supuestos/supuestos.json v0.8. No editar a mano: cambiar el JSON y regenerar.</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>MixTipos: proporción de personas de cada tipo dentro de su grupo (derivado de S04, corregido por raciones), sin TACC (S13, real), si es vianda y a qué fila va en E4 (D06), y la distribución de raciones por persona: P1Racion, P2Raciones, P3Raciones (S21, generado).</t>
+          <t>MixTipos: proporción de personas de cada tipo dentro de su grupo (derivado de S04, corregido por raciones), sin TACC (S13, real), si es vianda (informativo: todos hacen la misma fila) y la distribución de raciones por persona: P1Racion, P2Raciones, P3Raciones (S21, generado).</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Escenarios: E0 a E5 para cada perfil. PuestosBase y PuestosExtra son puestos de la fila general; el extra se habilita entre ExtraDesde_s y ExtraHasta_s (E2). FactorValidacion multiplica el tiempo de validación (E3, S24). FilasPorTipo = 1 en E4: se suma un puesto solo para viandas, con su propia fila (D06). Servidores = personas sirviendo (S22). CapacidadFilaServicio = 999 (sin límite) hasta que el referente estime S23.</t>
+          <t>Escenarios: E0 a E5 para cada perfil. PuestosBase y PuestosExtra son puestos de la caja, con una fila única; el extra se habilita entre ExtraDesde_s y ExtraHasta_s (E2). FactorValidacion multiplica el tiempo de validación (E3, S24). ProbVegetariano = proporción de personas con menú vegetariano (S27). Servidores = personas sirviendo, una de ellas a cargo de la comida vegetariana (S22). CapacidadFilaServicio = 999 (sin límite) hasta que el referente estime S23.</t>
         </is>
       </c>
     </row>
@@ -2900,20 +2900,20 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4</v>
+        <v>0.21</v>
       </c>
       <c r="F3" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="G3" t="n">
-        <v>5.42</v>
+        <v>21.47</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>lognormal2(0, 5, 0.4, getstream(activity))</t>
+          <t>lognormal2(0, 21, 0.21, getstream(activity))</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -2949,7 +2949,7 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="23" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
@@ -3000,7 +3000,7 @@
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
-          <t>FilasPorTipo</t>
+          <t>ProbVegetariano</t>
         </is>
       </c>
       <c r="J1" s="4" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Base: 1 puesto, fila única</t>
+          <t>Base: 1 puesto, 3 personas sirviendo</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3061,10 +3061,10 @@
         <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K2" t="n">
         <v>999</v>
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2 puestos, fila única</t>
+          <t>2 puestos, 3 personas sirviendo</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3111,10 +3111,10 @@
         <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="J3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K3" t="n">
         <v>999</v>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2 puestos de 12:00 a 13:30, fila única</t>
+          <t>2 puestos de 12:00 a 13:30, 3 personas sirviendo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3161,10 +3161,10 @@
         <v>1</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="J4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K4" t="n">
         <v>999</v>
@@ -3187,7 +3187,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1 puesto con validación por QR</t>
+          <t>1 puesto con validación por QR, 3 personas sirviendo</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3211,10 +3211,10 @@
         <v>0.6</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="J5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K5" t="n">
         <v>999</v>
@@ -3237,7 +3237,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2 puestos: fila de viandas y fila general</t>
+          <t>1 puesto, 4 personas sirviendo</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3261,10 +3261,10 @@
         <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>0.12</v>
       </c>
       <c r="J6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K6" t="n">
         <v>999</v>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2 puestos, fila única y 3 personas sirviendo</t>
+          <t>2 puestos, 4 personas sirviendo</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3311,10 +3311,10 @@
         <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="J7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K7" t="n">
         <v>999</v>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Base: 1 puesto, fila única</t>
+          <t>Base: 1 puesto, 3 personas sirviendo</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3361,10 +3361,10 @@
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K8" t="n">
         <v>999</v>
@@ -3387,7 +3387,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2 puestos, fila única</t>
+          <t>2 puestos, 3 personas sirviendo</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3411,10 +3411,10 @@
         <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="J9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" t="n">
         <v>999</v>
@@ -3437,7 +3437,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2 puestos de 12:00 a 13:30, fila única</t>
+          <t>2 puestos de 12:00 a 13:30, 3 personas sirviendo</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3461,10 +3461,10 @@
         <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="J10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K10" t="n">
         <v>999</v>
@@ -3487,7 +3487,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1 puesto con validación por QR</t>
+          <t>1 puesto con validación por QR, 3 personas sirviendo</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3511,10 +3511,10 @@
         <v>0.6</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="J11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
         <v>999</v>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2 puestos: fila de viandas y fila general</t>
+          <t>1 puesto, 4 personas sirviendo</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -3561,10 +3561,10 @@
         <v>1</v>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
+        <v>0.12</v>
       </c>
       <c r="J12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K12" t="n">
         <v>999</v>
@@ -3587,7 +3587,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2 puestos, fila única y 3 personas sirviendo</t>
+          <t>2 puestos, 4 personas sirviendo</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3611,10 +3611,10 @@
         <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="J13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13" t="n">
         <v>999</v>

</xml_diff>

<commit_message>
Servicio por ración de 15 a 20 s (mediana 17,3 s, sigma 0,09) en supuestos, tablas y guía
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/flexsim/inputs.xlsx
+++ b/flexsim/inputs.xlsx
@@ -2900,20 +2900,20 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>21</v>
+        <v>17.3</v>
       </c>
       <c r="E3" t="n">
-        <v>0.21</v>
+        <v>0.09</v>
       </c>
       <c r="F3" t="n">
-        <v>21</v>
+        <v>17.3</v>
       </c>
       <c r="G3" t="n">
-        <v>21.47</v>
+        <v>17.37</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>lognormal2(0, 21, 0.21, getstream(activity))</t>
+          <t>lognormal2(0, 17.3, 0.09, getstream(activity))</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">

</xml_diff>